<commit_message>
fix: varient to vairant
</commit_message>
<xml_diff>
--- a/param_config/param_data_naninovel.xlsx
+++ b/param_config/param_data_naninovel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】dev\param_config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】git仓库\param_config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A77C839-8678-46CA-9BAB-983CD2A7D98A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDB494C-3A88-4D69-8D65-7ED685A171EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" firstSheet="5" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Music" sheetId="8" r:id="rId1"/>
@@ -24,7 +24,7 @@
     <sheet name="Id" sheetId="1" r:id="rId9"/>
     <sheet name="Name" sheetId="5" r:id="rId10"/>
     <sheet name="Character" sheetId="11" r:id="rId11"/>
-    <sheet name="Varient" sheetId="16" r:id="rId12"/>
+    <sheet name="Variant" sheetId="16" r:id="rId12"/>
     <sheet name="Pose" sheetId="2" r:id="rId13"/>
     <sheet name="Tint" sheetId="18" r:id="rId14"/>
     <sheet name="Animation" sheetId="12" r:id="rId15"/>
@@ -507,6 +507,7 @@
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <xxl21:alternateUrls>
       <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
     </xxl21:alternateUrls>
     <sheetNames>
       <sheetName val="测试模版"/>
@@ -938,9 +939,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4D0EA6C-94B5-4B28-9D79-AE5F33D06CF7}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -978,9 +979,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{938A5E86-0F35-431D-B760-B491C7011A1E}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1018,9 +1019,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B366D178-7CDC-4708-83DB-8F05B13E7EF6}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1058,9 +1059,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{204E1CB4-0839-4C3B-A7A7-EACE42D226D8}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1090,9 +1091,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1146,9 +1147,9 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FCE18EF0-AEBE-4348-BCBF-A1A94009AC4C}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="4" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="4" customWidth="1"/>
     <col min="3" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
@@ -1194,9 +1195,9 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E58EBDF9-D3A0-47BB-830B-8DFDC52004A0}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1226,9 +1227,9 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7F2FB37-B05C-42DD-AD48-6F5711AA0F97}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1258,9 +1259,9 @@
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8BF32C34-7DB5-482B-A30F-C4A52DA2D4C1}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1290,9 +1291,9 @@
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EE5E455-8B28-43AD-99F6-BA5F70869328}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="4" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="4" customWidth="1"/>
     <col min="3" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
@@ -1346,9 +1347,9 @@
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B139D31-73BB-4244-8F5A-942E29743A69}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1394,9 +1395,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{966183FE-893C-4CE5-91A9-7B2DDB5030D5}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1434,9 +1435,9 @@
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69CF8993-2144-488C-A876-54C4032DB63D}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1490,9 +1491,9 @@
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD06AC-723F-4A84-9034-732CCFF1C997}">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1514,9 +1515,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9142AB7-47C3-437F-AB38-2468726F6E9E}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1554,9 +1555,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A521C93D-9983-4554-8EB8-0FE7DA0F0FDA}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="4" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="4" customWidth="1"/>
     <col min="3" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
@@ -1602,9 +1603,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6F9E9FB7-4439-4606-A4F6-AC47C23E9D2F}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1642,9 +1643,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{411C9431-5A00-4744-B00C-BA97A5030B47}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1698,9 +1699,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C90C90F-14F7-48DC-A223-3A21F823BBD9}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1738,9 +1739,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D0F9688-485C-4089-A924-659F7B17ED40}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
@@ -1778,9 +1779,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.5" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="2" width="40.6328125" style="1" customWidth="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
     <col min="3" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
``` feat(core): add AutoBlockTransition enum for automatic blocking transitions
Add new AutoBlockTransition enum with values for different types of
automatic indent transitions including New Scene, Partial Transition,
Character Transition, and Transition Block.
```
</commit_message>
<xml_diff>
--- a/param_config/param_data_naninovel.xlsx
+++ b/param_config/param_data_naninovel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】git仓库\param_config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CDB494C-3A88-4D69-8D65-7ED685A171EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBFF9D3-C2EE-4E5E-AD24-A9D183EEE613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="5" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="6" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Music" sheetId="8" r:id="rId1"/>
@@ -31,12 +31,13 @@
     <sheet name="Movie" sheetId="10" r:id="rId16"/>
     <sheet name="Dissolve" sheetId="21" r:id="rId17"/>
     <sheet name="Transition" sheetId="14" r:id="rId18"/>
-    <sheet name="TransitionType" sheetId="15" r:id="rId19"/>
-    <sheet name="Printer" sheetId="22" r:id="rId20"/>
-    <sheet name="基础参数模板" sheetId="4" r:id="rId21"/>
+    <sheet name="TransitionSub" sheetId="23" r:id="rId19"/>
+    <sheet name="TransitionType" sheetId="15" r:id="rId20"/>
+    <sheet name="Printer" sheetId="22" r:id="rId21"/>
+    <sheet name="基础参数模板" sheetId="4" r:id="rId22"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId22"/>
+    <externalReference r:id="rId23"/>
   </externalReferences>
   <definedNames>
     <definedName name="AmbienceList">OFFSET([1]参数表!$C$2,0,0,COUNTA([1]参数表!$C:$C)-1,1)</definedName>
@@ -72,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="108">
   <si>
     <t>ExcelParam</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -146,22 +147,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PartTransOnly</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>局部转场</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>PartTransNew</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>组合模块_新场景</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>转白</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -395,6 +384,126 @@
   </si>
   <si>
     <t>@blur power:0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>新场景</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NewScene</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>PartTrans</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>过渡局部转场</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PartTransBetween</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>转场组件</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>TransBlock</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>转场新场景</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>TransNewScene</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>过渡新场景</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>NewSceneBetween</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>局部转场开始</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>局部转场结束</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PartTransStart</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PartTransEnd</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>隐藏对话框</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>等待i0.5</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>等待i1</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>显示对话框</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>隐藏全部</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>√</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>局部转场长</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>PartTransLonger</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>隐藏立绘</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>立绘转场</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>过渡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开始</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>结束</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CharTrans</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开场</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -963,10 +1072,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -1038,7 +1147,7 @@
         <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1075,10 +1184,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1107,10 +1216,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1163,26 +1272,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>56</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1211,10 +1320,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -1243,10 +1352,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1275,10 +1384,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1290,51 +1399,204 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5EE5E455-8B28-43AD-99F6-BA5F70869328}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="40.6640625" style="4" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="3"/>
+    <col min="3" max="3" width="9" style="3"/>
+    <col min="4" max="9" width="9" style="4"/>
+    <col min="10" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>18</v>
+        <v>80</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="I17" s="4" t="s">
+        <v>98</v>
       </c>
     </row>
   </sheetData>
@@ -1345,44 +1607,60 @@
 </file>
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B139D31-73BB-4244-8F5A-942E29743A69}">
-  <dimension ref="A1:B4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7467A93B-8B97-40C6-9EB7-8194F72DDFFE}">
+  <dimension ref="A1:I5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="9" style="2"/>
+    <col min="1" max="2" width="40.6640625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="9" style="3"/>
+    <col min="4" max="9" width="9" style="4"/>
+    <col min="10" max="16384" width="9" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>37</v>
+      <c r="D1" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1419,10 +1697,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1433,6 +1711,54 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B139D31-73BB-4244-8F5A-942E29743A69}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69CF8993-2144-488C-A876-54C4032DB63D}">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
@@ -1451,34 +1777,34 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1488,7 +1814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD06AC-723F-4A84-9034-732CCFF1C997}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
@@ -1539,10 +1865,10 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1571,26 +1897,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1619,18 +1945,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1659,34 +1985,34 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1698,7 +2024,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C90C90F-14F7-48DC-A223-3A21F823BBD9}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
@@ -1715,18 +2041,26 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1755,18 +2089,18 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1795,10 +2129,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1811,10 +2145,10 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add camera processing capability and enhance character generator with animation configurations
</commit_message>
<xml_diff>
--- a/param_config/param_data_naninovel.xlsx
+++ b/param_config/param_data_naninovel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\视觉小说项目\【表格演出工具】git仓库\param_config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DBFF9D3-C2EE-4E5E-AD24-A9D183EEE613}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC4C3AD1-C099-4746-ABBE-D4C693CC3B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="6" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="11" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Music" sheetId="8" r:id="rId1"/>
@@ -34,10 +34,11 @@
     <sheet name="TransitionSub" sheetId="23" r:id="rId19"/>
     <sheet name="TransitionType" sheetId="15" r:id="rId20"/>
     <sheet name="Printer" sheetId="22" r:id="rId21"/>
-    <sheet name="基础参数模板" sheetId="4" r:id="rId22"/>
+    <sheet name="PrinterState" sheetId="24" r:id="rId22"/>
+    <sheet name="基础参数模板" sheetId="4" r:id="rId23"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId23"/>
+    <externalReference r:id="rId24"/>
   </externalReferences>
   <definedNames>
     <definedName name="AmbienceList">OFFSET([1]参数表!$C$2,0,0,COUNTA([1]参数表!$C:$C)-1,1)</definedName>
@@ -73,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="108">
   <si>
     <t>ExcelParam</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1760,7 +1761,39 @@
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69CF8993-2144-488C-A876-54C4032DB63D}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="9" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5EE41A1-0F0A-4C1D-8C8B-610809DF9616}">
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="40.6640625" style="1" customWidth="1"/>
@@ -1799,14 +1832,6 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1814,7 +1839,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54CD06AC-723F-4A84-9034-732CCFF1C997}">
   <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="11.4" x14ac:dyDescent="0.25"/>

</xml_diff>